<commit_message>
duration + chronic dis
</commit_message>
<xml_diff>
--- a/output/Tables/Best practice/prop_below_target.xlsx
+++ b/output/Tables/Best practice/prop_below_target.xlsx
@@ -383,13 +383,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>73.40214204598983</v>
+        <v>76.95457343962657</v>
       </c>
       <c r="C2">
-        <v>71.50260023584877</v>
+        <v>75.13348101488337</v>
       </c>
       <c r="D2">
-        <v>75.30168385613089</v>
+        <v>78.77566586436977</v>
       </c>
     </row>
     <row r="3">
@@ -399,13 +399,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>73.86226442315072</v>
+        <v>78.30544055203299</v>
       </c>
       <c r="C3">
-        <v>72.26635324425447</v>
+        <v>76.80025598809534</v>
       </c>
       <c r="D3">
-        <v>75.45817560204695</v>
+        <v>79.81062511597064</v>
       </c>
     </row>
     <row r="4">
@@ -415,13 +415,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>54.66542384971016</v>
+        <v>56.13449389326208</v>
       </c>
       <c r="C4">
-        <v>52.88909387827906</v>
+        <v>54.35907451144736</v>
       </c>
       <c r="D4">
-        <v>56.44175382114126</v>
+        <v>57.90991327507681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>